<commit_message>
QMD briefing mapped to new workflow
</commit_message>
<xml_diff>
--- a/outputs/public/briefings/cvd_case_fatality_2023_v1/workbook/bnr_cvd_case_fatality_2023_v1.xlsx
+++ b/outputs/public/briefings/cvd_case_fatality_2023_v1/workbook/bnr_cvd_case_fatality_2023_v1.xlsx
@@ -84,7 +84,7 @@
     <t>2023</t>
   </si>
   <si>
-    <t>2026-05-15</t>
+    <t>2026-08-07</t>
   </si>
   <si>
     <t>Data sheets, dataset metadata sheets, and variable metadata sheets</t>
@@ -243,9 +243,6 @@
     <t>v1</t>
   </si>
   <si>
-    <t>2026-05-06</t>
-  </si>
-  <si>
     <t>Ian Hambleton, Analyst</t>
   </si>
   <si>
@@ -276,7 +273,7 @@
     <t>CC BY 4.0 Attribution</t>
   </si>
   <si>
-    <t>Barbados National Registry approved cardiovascular registry extract (Jan 2010-Dec 2023)</t>
+    <t>bnr_cvd_input_case_fatality_202401_v01</t>
   </si>
   <si>
     <t>Barbados National Registry</t>
@@ -291,18 +288,21 @@
     <t>float</t>
   </si>
   <si>
+    <t>byte</t>
+  </si>
+  <si>
     <t>double</t>
   </si>
   <si>
     <t>display_format</t>
   </si>
   <si>
+    <t>%8.0g</t>
+  </si>
+  <si>
     <t>%9.0g</t>
   </si>
   <si>
-    <t>%8.0g</t>
-  </si>
-  <si>
     <t>%4.1f</t>
   </si>
   <si>
@@ -327,13 +327,13 @@
     <t>variable_label</t>
   </si>
   <si>
-    <t>CVD Event Type (AMI=2, Stroke=1)</t>
-  </si>
-  <si>
-    <t>Patient sex (1=female, 2=male)</t>
-  </si>
-  <si>
-    <t>Two year intervals between 2010 and 2023</t>
+    <t>CVD event type</t>
+  </si>
+  <si>
+    <t>Sex at birth</t>
+  </si>
+  <si>
+    <t>Two-year intervals between 2010 and 2023</t>
   </si>
   <si>
     <t>Number of events</t>
@@ -387,7 +387,7 @@
     <t xml:space="preserve">1=Female; 2=Male; </t>
   </si>
   <si>
-    <t xml:space="preserve">1=2010-2011; 2=2012-2013; 3=2014-2015; 4=2016-2017; 5=2018-2019; 6=2020-2021; 7=2022-2023; 8=2010-2011; 9=2012-2013; 10=2014-2015; 11=2016-2017; 12=2018-2019; 13=2020-2021; </t>
+    <t xml:space="preserve">1=2010-2011; 2=2012-2013; 3=2014-2015; 4=2016-2017; 5=2018-2019; 6=2020-2021; 7=2022-2023; 8=2012-2013; 9=2014-2015; 10=2016-2017; 11=2018-2019; 12=2020-2021; 13=2022-2023; </t>
   </si>
 </sst>
 </file>
@@ -1405,7 +1405,7 @@
         <v>30</v>
       </c>
       <c r="C17" t="s">
-        <v>33</v>
+        <v>34</v>
       </c>
       <c r="D17" s="1">
         <v>160</v>
@@ -1458,7 +1458,7 @@
         <v>30</v>
       </c>
       <c r="C18" t="s">
-        <v>34</v>
+        <v>35</v>
       </c>
       <c r="D18" s="1">
         <v>209</v>
@@ -1511,7 +1511,7 @@
         <v>30</v>
       </c>
       <c r="C19" t="s">
-        <v>35</v>
+        <v>36</v>
       </c>
       <c r="D19" s="1">
         <v>226</v>
@@ -1564,7 +1564,7 @@
         <v>30</v>
       </c>
       <c r="C20" t="s">
-        <v>36</v>
+        <v>37</v>
       </c>
       <c r="D20" s="1">
         <v>257</v>
@@ -1617,7 +1617,7 @@
         <v>30</v>
       </c>
       <c r="C21" t="s">
-        <v>37</v>
+        <v>38</v>
       </c>
       <c r="D21" s="1">
         <v>214</v>
@@ -1670,7 +1670,7 @@
         <v>30</v>
       </c>
       <c r="C22" t="s">
-        <v>38</v>
+        <v>39</v>
       </c>
       <c r="D22" s="1">
         <v>210</v>
@@ -1776,7 +1776,7 @@
         <v>31</v>
       </c>
       <c r="C24" t="s">
-        <v>33</v>
+        <v>34</v>
       </c>
       <c r="D24" s="1">
         <v>180</v>
@@ -1829,7 +1829,7 @@
         <v>31</v>
       </c>
       <c r="C25" t="s">
-        <v>34</v>
+        <v>35</v>
       </c>
       <c r="D25" s="1">
         <v>236</v>
@@ -1882,7 +1882,7 @@
         <v>31</v>
       </c>
       <c r="C26" t="s">
-        <v>35</v>
+        <v>36</v>
       </c>
       <c r="D26" s="1">
         <v>269</v>
@@ -1935,7 +1935,7 @@
         <v>31</v>
       </c>
       <c r="C27" t="s">
-        <v>36</v>
+        <v>37</v>
       </c>
       <c r="D27" s="1">
         <v>311</v>
@@ -1988,7 +1988,7 @@
         <v>31</v>
       </c>
       <c r="C28" t="s">
-        <v>37</v>
+        <v>38</v>
       </c>
       <c r="D28" s="1">
         <v>278</v>
@@ -2041,7 +2041,7 @@
         <v>31</v>
       </c>
       <c r="C29" t="s">
-        <v>38</v>
+        <v>39</v>
       </c>
       <c r="D29" s="1">
         <v>276</v>
@@ -2136,7 +2136,7 @@
         <v>58</v>
       </c>
       <c r="C4" t="s">
-        <v>75</v>
+        <v>22</v>
       </c>
     </row>
     <row r="5">
@@ -2147,7 +2147,7 @@
         <v>59</v>
       </c>
       <c r="C5" t="s">
-        <v>76</v>
+        <v>75</v>
       </c>
     </row>
     <row r="6">
@@ -2169,7 +2169,7 @@
         <v>61</v>
       </c>
       <c r="C7" t="s">
-        <v>77</v>
+        <v>76</v>
       </c>
     </row>
     <row r="8">
@@ -2180,7 +2180,7 @@
         <v>62</v>
       </c>
       <c r="C8" t="s">
-        <v>78</v>
+        <v>77</v>
       </c>
     </row>
     <row r="9">
@@ -2191,7 +2191,7 @@
         <v>63</v>
       </c>
       <c r="C9" t="s">
-        <v>79</v>
+        <v>78</v>
       </c>
     </row>
     <row r="10">
@@ -2213,7 +2213,7 @@
         <v>65</v>
       </c>
       <c r="C11" t="s">
-        <v>80</v>
+        <v>79</v>
       </c>
     </row>
     <row r="12">
@@ -2224,7 +2224,7 @@
         <v>66</v>
       </c>
       <c r="C12" t="s">
-        <v>81</v>
+        <v>80</v>
       </c>
     </row>
     <row r="13">
@@ -2235,7 +2235,7 @@
         <v>67</v>
       </c>
       <c r="C13" t="s">
-        <v>82</v>
+        <v>81</v>
       </c>
     </row>
     <row r="14">
@@ -2246,7 +2246,7 @@
         <v>68</v>
       </c>
       <c r="C14" t="s">
-        <v>83</v>
+        <v>82</v>
       </c>
     </row>
     <row r="15">
@@ -2257,7 +2257,7 @@
         <v>69</v>
       </c>
       <c r="C15" t="s">
-        <v>84</v>
+        <v>83</v>
       </c>
     </row>
     <row r="16">
@@ -2268,7 +2268,7 @@
         <v>70</v>
       </c>
       <c r="C16" t="s">
-        <v>85</v>
+        <v>84</v>
       </c>
     </row>
     <row r="17">
@@ -2279,7 +2279,7 @@
         <v>71</v>
       </c>
       <c r="C17" t="s">
-        <v>86</v>
+        <v>85</v>
       </c>
     </row>
     <row r="18">
@@ -2290,7 +2290,7 @@
         <v>72</v>
       </c>
       <c r="C18" t="s">
-        <v>87</v>
+        <v>86</v>
       </c>
     </row>
   </sheetData>
@@ -2307,10 +2307,10 @@
         <v>54</v>
       </c>
       <c r="B1" t="s">
+        <v>87</v>
+      </c>
+      <c r="C1" t="s">
         <v>88</v>
-      </c>
-      <c r="C1" t="s">
-        <v>89</v>
       </c>
       <c r="D1" t="s">
         <v>92</v>
@@ -2333,7 +2333,7 @@
         <v>26</v>
       </c>
       <c r="C2" t="s">
-        <v>90</v>
+        <v>89</v>
       </c>
       <c r="D2" t="s">
         <v>93</v>
@@ -2359,7 +2359,7 @@
         <v>90</v>
       </c>
       <c r="D3" t="s">
-        <v>94</v>
+        <v>93</v>
       </c>
       <c r="E3" t="s">
         <v>99</v>
@@ -2379,10 +2379,10 @@
         <v>32</v>
       </c>
       <c r="C4" t="s">
-        <v>90</v>
+        <v>89</v>
       </c>
       <c r="D4" t="s">
-        <v>93</v>
+        <v>94</v>
       </c>
       <c r="E4" t="s">
         <v>100</v>
@@ -2405,7 +2405,7 @@
         <v>91</v>
       </c>
       <c r="D5" t="s">
-        <v>93</v>
+        <v>94</v>
       </c>
       <c r="E5" t="s">
         <v>101</v>
@@ -2428,7 +2428,7 @@
         <v>91</v>
       </c>
       <c r="D6" t="s">
-        <v>94</v>
+        <v>93</v>
       </c>
       <c r="E6" t="s">
         <v>101</v>
@@ -2451,7 +2451,7 @@
         <v>91</v>
       </c>
       <c r="D7" t="s">
-        <v>94</v>
+        <v>93</v>
       </c>
       <c r="E7" t="s">
         <v>101</v>
@@ -2474,7 +2474,7 @@
         <v>91</v>
       </c>
       <c r="D8" t="s">
-        <v>94</v>
+        <v>93</v>
       </c>
       <c r="E8" t="s">
         <v>101</v>
@@ -2497,7 +2497,7 @@
         <v>91</v>
       </c>
       <c r="D9" t="s">
-        <v>94</v>
+        <v>93</v>
       </c>
       <c r="E9" t="s">
         <v>101</v>
@@ -2520,7 +2520,7 @@
         <v>91</v>
       </c>
       <c r="D10" t="s">
-        <v>94</v>
+        <v>93</v>
       </c>
       <c r="E10" t="s">
         <v>101</v>
@@ -2540,7 +2540,7 @@
         <v>46</v>
       </c>
       <c r="C11" t="s">
-        <v>90</v>
+        <v>89</v>
       </c>
       <c r="D11" t="s">
         <v>95</v>
@@ -2563,7 +2563,7 @@
         <v>47</v>
       </c>
       <c r="C12" t="s">
-        <v>90</v>
+        <v>89</v>
       </c>
       <c r="D12" t="s">
         <v>95</v>
@@ -2586,7 +2586,7 @@
         <v>48</v>
       </c>
       <c r="C13" t="s">
-        <v>90</v>
+        <v>89</v>
       </c>
       <c r="D13" t="s">
         <v>96</v>
@@ -2609,7 +2609,7 @@
         <v>49</v>
       </c>
       <c r="C14" t="s">
-        <v>90</v>
+        <v>89</v>
       </c>
       <c r="D14" t="s">
         <v>96</v>
@@ -2632,7 +2632,7 @@
         <v>50</v>
       </c>
       <c r="C15" t="s">
-        <v>90</v>
+        <v>89</v>
       </c>
       <c r="D15" t="s">
         <v>96</v>
@@ -2655,7 +2655,7 @@
         <v>51</v>
       </c>
       <c r="C16" t="s">
-        <v>90</v>
+        <v>89</v>
       </c>
       <c r="D16" t="s">
         <v>96</v>
@@ -2678,7 +2678,7 @@
         <v>52</v>
       </c>
       <c r="C17" t="s">
-        <v>90</v>
+        <v>89</v>
       </c>
       <c r="D17" t="s">
         <v>96</v>
@@ -2701,7 +2701,7 @@
         <v>53</v>
       </c>
       <c r="C18" t="s">
-        <v>90</v>
+        <v>89</v>
       </c>
       <c r="D18" t="s">
         <v>96</v>

</xml_diff>

<commit_message>
Briefing consolidation - updating key figures
</commit_message>
<xml_diff>
--- a/outputs/public/briefings/cvd_case_fatality_2023_v1/workbook/bnr_cvd_case_fatality_2023_v1.xlsx
+++ b/outputs/public/briefings/cvd_case_fatality_2023_v1/workbook/bnr_cvd_case_fatality_2023_v1.xlsx
@@ -84,7 +84,7 @@
     <t>2023</t>
   </si>
   <si>
-    <t>2026-08-07</t>
+    <t>2026-08-13</t>
   </si>
   <si>
     <t>Data sheets, dataset metadata sheets, and variable metadata sheets</t>
@@ -387,7 +387,7 @@
     <t xml:space="preserve">1=Female; 2=Male; </t>
   </si>
   <si>
-    <t xml:space="preserve">1=2010-2011; 2=2012-2013; 3=2014-2015; 4=2016-2017; 5=2018-2019; 6=2020-2021; 7=2022-2023; 8=2012-2013; 9=2014-2015; 10=2016-2017; 11=2018-2019; 12=2020-2021; 13=2022-2023; </t>
+    <t xml:space="preserve">1=2010-2011; 2=2012-2013; 3=2014-2015; 4=2016-2017; 5=2018-2019; 6=2020-2021; 7=2022-2023; </t>
   </si>
 </sst>
 </file>
@@ -1352,7 +1352,7 @@
         <v>30</v>
       </c>
       <c r="C16" t="s">
-        <v>39</v>
+        <v>33</v>
       </c>
       <c r="D16" s="1">
         <v>105</v>
@@ -1723,7 +1723,7 @@
         <v>31</v>
       </c>
       <c r="C23" t="s">
-        <v>39</v>
+        <v>33</v>
       </c>
       <c r="D23" s="1">
         <v>140</v>

</xml_diff>